<commit_message>
Added function to correct technologies parameters
</commit_message>
<xml_diff>
--- a/output/Summary.xlsx
+++ b/output/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -683,6 +683,208 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>output\20251121173006-1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>30960697.35755812</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4265505.792016438</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1936831.529638083</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6202337.321654522</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>24758360.0359036</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>30960697.35755812</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>112.1920001506805</v>
+      </c>
+      <c r="X3" t="n">
+        <v>30960697.35755811</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>30960697.35755812</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>3.725290298461914e-09</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AC3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>output\20251121180622-1</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>30980978.20867186</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4367103.613949267</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1965408.474573259</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6332512.088522526</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>24648466.12014933</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>30980978.20867186</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>118.3270001411438</v>
+      </c>
+      <c r="X4" t="n">
+        <v>30980978.20867186</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>30980978.20867186</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AC4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE4" t="n">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added mixer for HBfeed (still don0t know if it works)
</commit_message>
<xml_diff>
--- a/output/Summary.xlsx
+++ b/output/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1794,6 +1794,107 @@
         <v>1</v>
       </c>
       <c r="AE13" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>output\20251127154536-1</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>187529033.7359362</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4497480.441085723</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2013576.258318128</v>
+      </c>
+      <c r="F14" t="n">
+        <v>156600300</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6511056.69940385</v>
+      </c>
+      <c r="H14" t="n">
+        <v>156600300</v>
+      </c>
+      <c r="I14" t="n">
+        <v>24467674.42935357</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-49997.39282129705</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>187529033.7359362</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="n">
+        <v>18.83299994468689</v>
+      </c>
+      <c r="X14" t="n">
+        <v>187529033.7359362</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>187529033.7359362</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AC14" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE14" t="n">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new sim for ammonia with new nodes
seems to work
</commit_message>
<xml_diff>
--- a/output/Summary.xlsx
+++ b/output/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2097,6 +2097,309 @@
         <v>1</v>
       </c>
       <c r="AE16" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>output\20251205113843-1</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3696999.336956954</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.007158240613208921</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.007158240613208921</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3836999.009796476</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-139999.6799977628</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>3696999.336956954</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
+        <v>1.177999973297119</v>
+      </c>
+      <c r="X17" t="n">
+        <v>3676881.849305025</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>3696999.336956954</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>20117.48765192879</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AC17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>output\20251205133221-1</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>64748274.98479408</v>
+      </c>
+      <c r="C18" t="n">
+        <v>11582708.18136209</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.234020655272847</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3926754.62290082</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>15509462.80426291</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.234020655272847</v>
+      </c>
+      <c r="I18" t="n">
+        <v>49238811.94651051</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>64748274.98479408</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="n">
+        <v>83.45899987220764</v>
+      </c>
+      <c r="X18" t="n">
+        <v>64748274.98479399</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>64748274.98479408</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>8.940696716308594e-08</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AC18" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>output\20251205135606-1</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>64762961.79300305</v>
+      </c>
+      <c r="C19" t="n">
+        <v>11758430.61511528</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.2385114218090135</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3992938.368812331</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>15751368.98392761</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.2385114218090135</v>
+      </c>
+      <c r="I19" t="n">
+        <v>49011592.57056402</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>64762961.79300305</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" t="n">
+        <v>159.1280000209808</v>
+      </c>
+      <c r="X19" t="n">
+        <v>64762961.79300298</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>64762961.79300305</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>6.705522537231445e-08</v>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AC19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE19" t="n">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new sim with SMR, but noticed problem with carriers demands
</commit_message>
<xml_diff>
--- a/output/Summary.xlsx
+++ b/output/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE19"/>
+  <dimension ref="A1:AE20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2400,6 +2400,107 @@
         <v>1</v>
       </c>
       <c r="AE19" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>output\20251205144145-1</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>64713563.74372575</v>
+      </c>
+      <c r="C20" t="n">
+        <v>11510221.19699504</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.2346726031689292</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3919016.830410321</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>15429238.02740537</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2346726031689292</v>
+      </c>
+      <c r="I20" t="n">
+        <v>49284325.48164778</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>64713563.74372575</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" t="n">
+        <v>106.3980000019073</v>
+      </c>
+      <c r="X20" t="n">
+        <v>64713563.74372575</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>64713563.74372575</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>7.450580596923828e-09</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AC20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE20" t="n">
         <v>-1</v>
       </c>
     </row>

</xml_diff>